<commit_message>
Fix QA Checks: Debt Payoff references corrected
All 6 models had QA Debt Payoff checks pointing to wrong rows:

| Model | Before | After | Row Label |
|-------|--------|-------|-----------|
| Peaker | K91 (Taxes) | K103 (Ending Balance) | ✓ |
| SolarBESS | N81 (Taxes) | N91 (Ending Balance) | ✓ |
| Transmission | N84 (EBIT) | N94 (Ending Balance) | ✓ |
| Midstream | I78 (CFADS) | I88 (Ending Balance) | ✓ |
| Wind | E90+D59 (Interest+Header) | E93+D62 (EndBal+Tenor) | ✓ |

All fixes propagated to corresponding Drill files.
All QA checks now verified to reference correct cells.

ZIP SHA256: 915ecaff3f965a2a62a9259822e076f1e54152056867d379ca4cc83e738f440a
</commit_message>
<xml_diff>
--- a/deliverables/deliverables-20260120-0030/Drill_2_Peaker.xlsx
+++ b/deliverables/deliverables-20260120-0030/Drill_2_Peaker.xlsx
@@ -3026,7 +3026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N160"/>
+  <dimension ref="A1:N144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3447,7 +3447,7 @@
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="10">
-        <f>IF(K91&lt;1,"PASS","FAIL")</f>
+        <f>IF(K103&lt;1,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
@@ -3474,7 +3474,6 @@
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="10" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -6468,22 +6467,6 @@
       <c r="C144" s="6" t="n"/>
       <c r="D144" s="31" t="n"/>
     </row>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="D7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>